<commit_message>
Update landing and clean legacy frontend assets
</commit_message>
<xml_diff>
--- a/public/modelos/modelo-completo.xlsx
+++ b/public/modelos/modelo-completo.xlsx
@@ -1,58 +1,173 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Produtos" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Produtos" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Como preencher" state="visible" r:id="rId5"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+  <si>
+    <t>Código</t>
+  </si>
+  <si>
+    <t>Nome do Produto</t>
+  </si>
+  <si>
+    <t>Preço</t>
+  </si>
+  <si>
+    <t>Descrição</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Variações</t>
+  </si>
+  <si>
+    <t>COP-001</t>
+  </si>
+  <si>
+    <t>Copo da Felicidade</t>
+  </si>
+  <si>
+    <t>12,00</t>
+  </si>
+  <si>
+    <t>Copo 200ml recheado com cremes especiais</t>
+  </si>
+  <si>
+    <t>Sobremesas</t>
+  </si>
+  <si>
+    <t>Supremo Morango:12, Supremo Nutella:14, Dois Amores:11, Ouro Branco:13, Maracujá:12</t>
+  </si>
+  <si>
+    <t>BOL-001</t>
+  </si>
+  <si>
+    <t>Bolo Personalizado</t>
+  </si>
+  <si>
+    <t>85,00</t>
+  </si>
+  <si>
+    <t>Massa branca ou cacau 50% com recheio escolhido</t>
+  </si>
+  <si>
+    <t>Bolos</t>
+  </si>
+  <si>
+    <t>10cm:85, 15cm:120, 20cm:160, 25cm:220, 30cm:300</t>
+  </si>
+  <si>
+    <t>Passo</t>
+  </si>
+  <si>
+    <t>Orientação</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Use esta planilha para preencher o Modelo completo do ZapCatálogo.</t>
+  </si>
+  <si>
+    <t>Cada linha é um produto.</t>
+  </si>
+  <si>
+    <t>Preço pode ser escrito como 12,00 ou 12.00.</t>
+  </si>
+  <si>
+    <t>Categoria é o grupo do produto.</t>
+  </si>
+  <si>
+    <t>Variações são opções separadas por vírgula.</t>
+  </si>
+  <si>
+    <t>Para variações com preço diferente, use: Supremo Morango:12, Supremo Nutella:14, Dois Amores:11</t>
+  </si>
+  <si>
+    <t>Código é opcional, mas recomendado para atualizar depois sem perder imagens.</t>
+  </si>
+  <si>
+    <t>Não apague os nomes das colunas.</t>
+  </si>
+  <si>
+    <t>Não mescle células.</t>
+  </si>
+  <si>
+    <t>Não coloque imagem dentro da planilha. Imagens são enviadas depois no sistema.</t>
+  </si>
+  <si>
+    <t>Exemplo</t>
+  </si>
+  <si>
+    <t>Supremo Morango:12, Supremo Nutella:14</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF128C7E"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF128C7E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6FFFA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -60,18 +175,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0F766E"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF0F766E"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF0F766E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF0F766E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE5E7EB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,60 +570,191 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="19.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Código</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Nome do Produto</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Preço</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Descrição</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Categoria</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Variações</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>CAM-001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Camiseta Polo</v>
-      </c>
-      <c r="C2" t="str">
-        <v>89,90</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Malha piquet azul</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Camisetas</v>
-      </c>
-      <c r="F2" t="str">
-        <v>P, M, G, GG</v>
+    <row r="1" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="100" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>8</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove code column from spreadsheet models
</commit_message>
<xml_diff>
--- a/public/modelos/modelo-completo.xlsx
+++ b/public/modelos/modelo-completo.xlsx
@@ -12,10 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
-  <si>
-    <t>Código</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>Nome do Produto</t>
   </si>
@@ -32,9 +29,6 @@
     <t>Variações</t>
   </si>
   <si>
-    <t>COP-001</t>
-  </si>
-  <si>
     <t>Copo da Felicidade</t>
   </si>
   <si>
@@ -50,9 +44,6 @@
     <t>Supremo Morango:12, Supremo Nutella:14, Dois Amores:11, Ouro Branco:13, Maracujá:12</t>
   </si>
   <si>
-    <t>BOL-001</t>
-  </si>
-  <si>
     <t>Bolo Personalizado</t>
   </si>
   <si>
@@ -68,40 +59,76 @@
     <t>10cm:85, 15cm:120, 20cm:160, 25cm:220, 30cm:300</t>
   </si>
   <si>
+    <t>Torta de Limão</t>
+  </si>
+  <si>
+    <t>39,90</t>
+  </si>
+  <si>
+    <t>Torta cremosa com base crocante</t>
+  </si>
+  <si>
+    <t>Fatia:39,90, Inteira:149,90</t>
+  </si>
+  <si>
+    <t>Combo Família</t>
+  </si>
+  <si>
+    <t>129,90</t>
+  </si>
+  <si>
+    <t>Lanche com acompanhamento e bebida</t>
+  </si>
+  <si>
+    <t>Lanches</t>
+  </si>
+  <si>
+    <t>Padrão:129,90, Especial:149,90</t>
+  </si>
+  <si>
     <t>Passo</t>
   </si>
   <si>
     <t>Orientação</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Use esta planilha para preencher o Modelo completo do ZapCatálogo.</t>
-  </si>
-  <si>
-    <t>Cada linha é um produto.</t>
-  </si>
-  <si>
-    <t>Preço pode ser escrito como 12,00 ou 12.00.</t>
-  </si>
-  <si>
-    <t>Categoria é o grupo do produto.</t>
-  </si>
-  <si>
-    <t>Variações são opções separadas por vírgula.</t>
-  </si>
-  <si>
-    <t>Para variações com preço diferente, use: Supremo Morango:12, Supremo Nutella:14, Dois Amores:11</t>
-  </si>
-  <si>
-    <t>Código é opcional, mas recomendado para atualizar depois sem perder imagens.</t>
-  </si>
-  <si>
-    <t>Não apague os nomes das colunas.</t>
-  </si>
-  <si>
-    <t>Não mescle células.</t>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Modelo mais completo, com mais exemplos para quem quer copiar e preencher rápido.</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Cada linha vira um produto no catálogo.</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Use os modelos prontos para não errar as colunas.</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Se a variação não tiver preço, o catálogo usa o preço base do produto.</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Para atualizar produtos depois, mantenha o mesmo nome do produto. Assim suas imagens continuam vinculadas automaticamente.</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Não apague os nomes das colunas nem mescle células.</t>
+  </si>
+  <si>
+    <t>7</t>
   </si>
   <si>
     <t>Não coloque imagem dentro da planilha. Imagens são enviadas depois no sistema.</t>
@@ -110,7 +137,7 @@
     <t>Exemplo</t>
   </si>
   <si>
-    <t>Supremo Morango:12, Supremo Nutella:14</t>
+    <t>Supremo Morango:12, Supremo Nutella:14, Dois Amores:11</t>
   </si>
 </sst>
 </file>
@@ -139,7 +166,7 @@
       <color rgb="FF128C7E"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -149,11 +176,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF128C7E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -209,28 +231,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -571,18 +587,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="76" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="76" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -598,48 +613,73 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" ht="48" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2" t="s">
+    </row>
+    <row r="3" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" ht="48" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
+    </row>
+    <row r="4" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>17</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -650,107 +690,83 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>19</v>
+    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>21</v>
+      <c r="A2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="6">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>22</v>
+      <c r="A3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="6">
-        <v>2</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>23</v>
+      <c r="A4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="6">
-        <v>3</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>24</v>
+      <c r="A5" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="6">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>25</v>
+      <c r="A6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="6">
-        <v>5</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>26</v>
+      <c r="A7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
-        <v>6</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>27</v>
+      <c r="A8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
-        <v>7</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
-        <v>8</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
-        <v>9</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>32</v>
+      <c r="A9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>